<commit_message>
Updated LR with dropped missing value
</commit_message>
<xml_diff>
--- a/Model/LR/aqi_metrics_lr.xlsx
+++ b/Model/LR/aqi_metrics_lr.xlsx
@@ -414,13 +414,13 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>0.8532111981561211</v>
+        <v>0.8599206949088777</v>
       </c>
       <c r="C2">
-        <v>0.5823754789272031</v>
+        <v>0.5862068965517241</v>
       </c>
       <c r="D2">
-        <v>39.50191570881226</v>
+        <v>39.82120051085569</v>
       </c>
       <c r="E2">
         <v>261</v>
@@ -431,13 +431,13 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>1.130959666584914</v>
+        <v>1.062029649653994</v>
       </c>
       <c r="C3">
-        <v>0.8372093023255814</v>
+        <v>0.7558139534883721</v>
       </c>
       <c r="D3">
-        <v>48.81782945736434</v>
+        <v>39.80620155038761</v>
       </c>
       <c r="E3">
         <v>86</v>
@@ -448,16 +448,16 @@
         <v>6</v>
       </c>
       <c r="B4">
-        <v>0.4224200062852577</v>
+        <v>0.6226998490772391</v>
       </c>
       <c r="C4">
-        <v>0.1784386617100372</v>
+        <v>0.3775510204081632</v>
       </c>
       <c r="D4">
-        <v>10.78066914498141</v>
+        <v>28.48639455782313</v>
       </c>
       <c r="E4">
-        <v>269</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>